<commit_message>
Complete CO2 extension: update bulk BIPs, main runner options, and TIP calibration utilities
</commit_message>
<xml_diff>
--- a/config/MixtureData.xlsx
+++ b/config/MixtureData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Files\Matlab - Old\Sat_press\Dew point with Mineralogy\Pdew - o1 Version - Tenth version (Combined delta_Tc and Pdew)\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Files\Matlab - Old\Sat_press\Dew point with Mineralogy\Pdew - o1 Version - Tenth version (Combined delta_Tc and Pdew)\confined-thermo-eos\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1331373E-58E3-4F38-A9BF-228623A6B5E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E2CBDB9-9891-40F6-8753-E1FA2504BDAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Comp_Props" sheetId="12" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="67">
   <si>
     <t>Tc</t>
   </si>
@@ -227,6 +227,21 @@
   </si>
   <si>
     <t>Core</t>
+  </si>
+  <si>
+    <t>CO2</t>
+  </si>
+  <si>
+    <t>CO2-C1-nC8</t>
+  </si>
+  <si>
+    <t>[0.1,0.828,0.072]</t>
+  </si>
+  <si>
+    <t>CO2-C1-nC5</t>
+  </si>
+  <si>
+    <t>[0.15,0.7,0.15]</t>
   </si>
 </sst>
 </file>
@@ -567,10 +582,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33088355-66E5-4C2D-B80E-F792D01120EE}">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>26</v>
       </c>
@@ -605,7 +620,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -640,7 +655,7 @@
         <v>1.9400000000000002E-21</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -675,7 +690,7 @@
         <v>1.9999999999999998E-21</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -710,7 +725,7 @@
         <v>2.045E-21</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -744,6 +759,39 @@
       <c r="K5" s="1">
         <v>2.075E-21</v>
       </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B6">
+        <v>304.12799999999999</v>
+      </c>
+      <c r="C6" s="1">
+        <v>7377300</v>
+      </c>
+      <c r="D6">
+        <v>0.22394</v>
+      </c>
+      <c r="E6">
+        <v>44.01</v>
+      </c>
+      <c r="G6">
+        <v>78</v>
+      </c>
+      <c r="I6">
+        <v>5.0999999999999997E-2</v>
+      </c>
+      <c r="J6" s="1">
+        <v>3.9410000000000001E-10</v>
+      </c>
+      <c r="K6">
+        <v>3.0374248508930569E-21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -752,88 +800,123 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EC5FDCA-02AD-4494-B9AC-9328D27B8D8B}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C1" t="s">
         <v>8</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>9</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>10</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>0.1</v>
+      </c>
+      <c r="D2">
+        <v>0.44030000000000002</v>
+      </c>
+      <c r="E2">
+        <v>0.32190000000000002</v>
+      </c>
+      <c r="F2">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B2">
-        <v>0</v>
-      </c>
-      <c r="C2">
+      <c r="B3">
+        <v>0.1</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
         <v>1.2022E-2</v>
       </c>
-      <c r="D2">
+      <c r="E3">
         <v>1.5573E-2</v>
       </c>
-      <c r="E2">
+      <c r="F3">
         <v>3.9320000000000001E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>9</v>
       </c>
-      <c r="B3">
+      <c r="B4">
+        <v>0.44030000000000002</v>
+      </c>
+      <c r="C4">
         <v>1.2022E-2</v>
       </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-      <c r="E3">
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
         <v>8.9820000000000004E-3</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>10</v>
       </c>
-      <c r="B4">
+      <c r="B5">
+        <v>0.32190000000000002</v>
+      </c>
+      <c r="C5">
         <v>1.5573E-2</v>
       </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>11</v>
       </c>
-      <c r="B5">
+      <c r="B6">
+        <v>0.13</v>
+      </c>
+      <c r="C6">
         <v>3.9320000000000001E-2</v>
       </c>
-      <c r="C5">
+      <c r="D6">
         <v>8.9820000000000004E-3</v>
       </c>
-      <c r="D5">
-        <v>0</v>
-      </c>
-      <c r="E5">
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
         <v>0</v>
       </c>
     </row>
@@ -1070,7 +1153,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29E1C41D-40BE-4570-8BED-FFFB506E8018}">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1383,6 +1466,58 @@
       </c>
       <c r="H12">
         <v>142</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>63</v>
+      </c>
+      <c r="B13" t="s">
+        <v>64</v>
+      </c>
+      <c r="C13">
+        <v>4126</v>
+      </c>
+      <c r="D13" t="s">
+        <v>44</v>
+      </c>
+      <c r="E13">
+        <v>4261</v>
+      </c>
+      <c r="F13">
+        <v>4261</v>
+      </c>
+      <c r="G13">
+        <v>135</v>
+      </c>
+      <c r="H13">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>65</v>
+      </c>
+      <c r="B14" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14">
+        <v>2701</v>
+      </c>
+      <c r="D14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E14">
+        <v>2770</v>
+      </c>
+      <c r="F14">
+        <v>2770</v>
+      </c>
+      <c r="G14">
+        <v>69</v>
+      </c>
+      <c r="H14">
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>